<commit_message>
API Automation Test Suite Added
</commit_message>
<xml_diff>
--- a/ParaBankAutomationFramework/target/classes/ParaBank-TestData/ParaBank-TestDataExcelSheet.xlsx
+++ b/ParaBankAutomationFramework/target/classes/ParaBank-TestData/ParaBank-TestDataExcelSheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="29">
   <si>
     <t>password</t>
   </si>
@@ -88,21 +88,6 @@
     <t>InitialAccountID</t>
   </si>
   <si>
-    <t>15231</t>
-  </si>
-  <si>
-    <t>15342</t>
-  </si>
-  <si>
-    <t>15453</t>
-  </si>
-  <si>
-    <t>thomas</t>
-  </si>
-  <si>
-    <t>dom</t>
-  </si>
-  <si>
     <t>16230</t>
   </si>
   <si>
@@ -110,6 +95,12 @@
   </si>
   <si>
     <t>16452</t>
+  </si>
+  <si>
+    <t>tom</t>
+  </si>
+  <si>
+    <t>jerry</t>
   </si>
 </sst>
 </file>
@@ -493,12 +484,12 @@
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="23.7109375"/>
-    <col min="2" max="2" customWidth="true" width="28.42578125"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -509,7 +500,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -517,7 +508,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -525,7 +516,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -533,7 +524,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -541,7 +532,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1">
@@ -549,7 +540,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="1">
@@ -557,7 +548,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="1">
@@ -565,7 +556,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -573,7 +564,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -581,7 +572,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -589,11 +580,11 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s" s="0">
-        <v>30</v>
+      <c r="B12" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -633,7 +624,7 @@
         <v>23</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -650,7 +641,7 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s" s="0">
+      <c r="A20" t="s">
         <v>2</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -658,7 +649,7 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s" s="0">
+      <c r="A21" t="s">
         <v>3</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -666,7 +657,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s" s="0">
+      <c r="A22" t="s">
         <v>1</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -674,7 +665,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s" s="0">
+      <c r="A23" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -682,7 +673,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s" s="0">
+      <c r="A24" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -693,8 +684,8 @@
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B25" t="s" s="0">
-        <v>31</v>
+      <c r="B25" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>